<commit_message>
add DMM readings interface
</commit_message>
<xml_diff>
--- a/API_Short.xlsx
+++ b/API_Short.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cbwhitt\Documents\Collin B Whittaker\Research\DARPA Pitch Day\Remote Control DAQ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marksta\Documents\Projects\DARPA Diffusion Control\controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23806455-EEBA-4EDA-AE55-433C86777BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A90183-57C4-4B56-9AEE-F206B3B16289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Commands" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="80">
   <si>
     <t>Name</t>
   </si>
@@ -386,6 +386,9 @@
 4:"Status",
 5:"Remote"
 &gt;</t>
+  </si>
+  <si>
+    <t>DMM Get Readings</t>
   </si>
 </sst>
 </file>
@@ -763,18 +766,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E79977-5DE8-43D3-9E1F-0C46D71E498D}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="31.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="99.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="33.42578125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="21.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="99.54296875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.453125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -791,7 +794,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>16</v>
       </c>
@@ -808,7 +811,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>17</v>
       </c>
@@ -825,7 +828,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>18</v>
       </c>
@@ -842,7 +845,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>19</v>
       </c>
@@ -859,7 +862,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>24</v>
       </c>
@@ -876,7 +879,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>25</v>
       </c>
@@ -893,7 +896,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>26</v>
       </c>
@@ -910,7 +913,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>27</v>
       </c>
@@ -927,7 +930,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>28</v>
       </c>
@@ -944,7 +947,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="116" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>32</v>
       </c>
@@ -961,7 +964,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>33</v>
       </c>
@@ -978,7 +981,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>34</v>
       </c>
@@ -995,7 +998,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>35</v>
       </c>
@@ -1012,7 +1015,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>36</v>
       </c>
@@ -1027,6 +1030,14 @@
       </c>
       <c r="E15" s="1" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="1">
+        <v>49</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1037,14 +1048,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90851A12-AFFB-4458-8046-60B55AA1BCAE}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
-    <col min="2" max="2" width="144.85546875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="144.81640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1052,7 +1063,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -1060,7 +1071,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>53</v>
       </c>
@@ -1068,7 +1079,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>54</v>
       </c>
@@ -1076,7 +1087,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>55</v>
       </c>
@@ -1084,7 +1095,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>58</v>
       </c>
@@ -1092,7 +1103,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="180" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>60</v>
       </c>
@@ -1100,7 +1111,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="225" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="217.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>62</v>
       </c>
@@ -1108,7 +1119,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>64</v>
       </c>
@@ -1116,7 +1127,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>66</v>
       </c>
@@ -1124,7 +1135,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>33</v>
       </c>
@@ -1132,7 +1143,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1140,7 +1151,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>69</v>
       </c>
@@ -1148,7 +1159,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>70</v>
       </c>
@@ -1156,7 +1167,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="90" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>71</v>
       </c>

</xml_diff>

<commit_message>
implemented oscope config and calibration
</commit_message>
<xml_diff>
--- a/API_Short.xlsx
+++ b/API_Short.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marksta\Documents\Projects\DARPA Diffusion Control\controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6119C290-5B52-4248-A52D-5AAF4C20C65E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECCD2FD-ABCC-4517-BF79-336E389C44A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
   </bookViews>
   <sheets>
     <sheet name="Commands" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="87">
   <si>
     <t>Name</t>
   </si>
@@ -403,6 +403,18 @@
     <t>Cluster{
 "Current": double
 }</t>
+  </si>
+  <si>
+    <t>Oscope Configuration</t>
+  </si>
+  <si>
+    <t>Oscope config</t>
+  </si>
+  <si>
+    <t>Array [Cluster{
+"Label": str,
+"Collect_Waveform": bool,
+}]</t>
   </si>
 </sst>
 </file>
@@ -780,7 +792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E79977-5DE8-43D3-9E1F-0C46D71E498D}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.453125" style="1" customWidth="1"/>
@@ -1063,6 +1075,14 @@
         <v>81</v>
       </c>
     </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="1">
+        <v>42</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1070,11 +1090,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90851A12-AFFB-4458-8046-60B55AA1BCAE}">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
-    <col min="2" max="2" width="144.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.54296875" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
@@ -1206,6 +1226,14 @@
         <v>83</v>
       </c>
     </row>
+    <row r="17" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
first pass oscope range setting implementation
</commit_message>
<xml_diff>
--- a/API_Short.xlsx
+++ b/API_Short.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marksta\Documents\Projects\DARPA Diffusion Control\controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECCD2FD-ABCC-4517-BF79-336E389C44A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92215907-9B45-49F5-9B89-86EEB8CC0A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
   </bookViews>
@@ -413,6 +413,8 @@
   <si>
     <t>Array [Cluster{
 "Label": str,
+"Range": double,
+"Offset": double,
 "Collect_Waveform": bool,
 }]</t>
   </si>
@@ -1226,7 +1228,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>84</v>
       </c>

</xml_diff>

<commit_message>
refactor labview control to automatically pack and unpack
</commit_message>
<xml_diff>
--- a/API_Short.xlsx
+++ b/API_Short.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marksta\Documents\Projects\DARPA Diffusion Control\controls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2307F28-EC0C-4494-8299-19707294CA3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA9C47C-4968-4DC0-A0F7-CFA001E51F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A0352D46-BEC4-44D9-A019-89A612CE3CE9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="90">
   <si>
     <t>Name</t>
   </si>
@@ -411,11 +411,28 @@
     <t>Oscope config</t>
   </si>
   <si>
-    <t>Array [Cluster{
+    <t>Cluster{
+"Range": double,
+"Reference": enum (unsigned byte).
+"Position": double,
+}</t>
+  </si>
+  <si>
+    <t>Enum: 0: left, 1: center, 2: right
+Typically send 1</t>
+  </si>
+  <si>
+    <t>Cluster{
+"TimeBase": OscopeTimeBase,
+"Channels": Array [Cluster{
 "Label": str,
 "Range": double,
 "Collect_Waveform": bool,
-}]</t>
+}]
+}</t>
+  </si>
+  <si>
+    <t>OscopeTimeBase</t>
   </si>
 </sst>
 </file>
@@ -1091,12 +1108,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90851A12-AFFB-4458-8046-60B55AA1BCAE}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.54296875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.1796875" style="1"/>
+    <col min="3" max="3" width="28.81640625" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.1796875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -1227,12 +1245,23 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" ht="116" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A18" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>86</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>